<commit_message>
quité correo automático de momento
</commit_message>
<xml_diff>
--- a/data/enobnu/calendario.xlsx
+++ b/data/enobnu/calendario.xlsx
@@ -596,7 +596,7 @@
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
@@ -636,7 +636,7 @@
       <c r="H3" s="5" t="inlineStr"/>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr"/>
@@ -676,7 +676,7 @@
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
@@ -720,7 +720,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
@@ -764,7 +764,7 @@
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
@@ -804,7 +804,7 @@
       <c r="H7" s="5" t="inlineStr"/>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
@@ -848,7 +848,7 @@
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
@@ -888,7 +888,7 @@
       <c r="H9" s="5" t="inlineStr"/>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr"/>
@@ -928,7 +928,7 @@
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
@@ -968,7 +968,7 @@
       <c r="H11" s="5" t="inlineStr"/>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr"/>
@@ -1008,7 +1008,7 @@
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
@@ -1048,7 +1048,7 @@
       <c r="H13" s="5" t="inlineStr"/>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr"/>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1136,7 +1136,7 @@
       <c r="H15" s="5" t="inlineStr"/>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr"/>
@@ -1176,7 +1176,7 @@
       <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
@@ -1216,7 +1216,7 @@
       <c r="H17" s="5" t="inlineStr"/>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr"/>
@@ -1256,7 +1256,7 @@
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
@@ -1344,7 +1344,7 @@
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
@@ -1384,7 +1384,7 @@
       <c r="H21" s="5" t="inlineStr"/>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr"/>
@@ -1424,7 +1424,7 @@
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr"/>
@@ -1464,7 +1464,7 @@
       <c r="H23" s="5" t="inlineStr"/>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr"/>
@@ -1504,7 +1504,7 @@
       <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr"/>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
@@ -1592,7 +1592,7 @@
       <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
@@ -1632,7 +1632,7 @@
       <c r="H27" s="5" t="inlineStr"/>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr"/>
@@ -1672,7 +1672,7 @@
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
@@ -1760,7 +1760,7 @@
       <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
@@ -1800,7 +1800,7 @@
       <c r="H31" s="5" t="inlineStr"/>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr"/>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -1888,7 +1888,7 @@
       <c r="H33" s="5" t="inlineStr"/>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr"/>
@@ -1928,7 +1928,7 @@
       <c r="H34" s="9" t="inlineStr"/>
       <c r="I34" s="9" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J34" s="9" t="inlineStr">
@@ -1972,7 +1972,7 @@
       <c r="H35" s="9" t="inlineStr"/>
       <c r="I35" s="9" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J35" s="9" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -2064,7 +2064,7 @@
       <c r="H37" s="5" t="inlineStr"/>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr"/>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>JCS</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -2152,7 +2152,7 @@
       <c r="H39" s="5" t="inlineStr"/>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>JM, MB, VB</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr"/>
@@ -2232,7 +2232,7 @@
       <c r="H41" s="5" t="inlineStr"/>
       <c r="I41" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J41" s="5" t="inlineStr"/>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
@@ -2400,7 +2400,7 @@
       <c r="H45" s="12" t="inlineStr"/>
       <c r="I45" s="12" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J45" s="12" t="inlineStr">
@@ -2484,7 +2484,7 @@
       <c r="H47" s="5" t="inlineStr"/>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr"/>
@@ -2564,7 +2564,7 @@
       <c r="H49" s="5" t="inlineStr"/>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J49" s="5" t="inlineStr"/>
@@ -2644,7 +2644,7 @@
       <c r="H51" s="5" t="inlineStr"/>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr"/>
@@ -2732,7 +2732,7 @@
       <c r="H53" s="12" t="inlineStr"/>
       <c r="I53" s="12" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J53" s="12" t="inlineStr">
@@ -2816,7 +2816,7 @@
       <c r="H55" s="5" t="inlineStr"/>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr"/>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
@@ -2984,7 +2984,7 @@
       <c r="H59" s="5" t="inlineStr"/>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr"/>
@@ -3064,7 +3064,7 @@
       <c r="H61" s="5" t="inlineStr"/>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J61" s="5" t="inlineStr"/>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J63" s="5" t="inlineStr">
@@ -3232,7 +3232,7 @@
       <c r="H65" s="5" t="inlineStr"/>
       <c r="I65" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J65" s="5" t="inlineStr"/>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="I67" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J67" s="5" t="inlineStr">
@@ -3400,7 +3400,7 @@
       <c r="H69" s="5" t="inlineStr"/>
       <c r="I69" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J69" s="5" t="inlineStr"/>
@@ -3488,7 +3488,7 @@
       <c r="H71" s="5" t="inlineStr"/>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J71" s="5" t="inlineStr"/>
@@ -3572,7 +3572,7 @@
       <c r="H73" s="9" t="inlineStr"/>
       <c r="I73" s="9" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J73" s="9" t="inlineStr">
@@ -3664,7 +3664,7 @@
       <c r="H75" s="5" t="inlineStr"/>
       <c r="I75" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J75" s="5" t="inlineStr"/>
@@ -3752,7 +3752,7 @@
       <c r="H77" s="5" t="inlineStr"/>
       <c r="I77" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>NV, RM, SM</t>
         </is>
       </c>
       <c r="J77" s="5" t="inlineStr"/>
@@ -3792,7 +3792,7 @@
       <c r="H78" s="2" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr"/>
@@ -3832,7 +3832,7 @@
       <c r="H79" s="5" t="inlineStr"/>
       <c r="I79" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J79" s="5" t="inlineStr"/>
@@ -3872,7 +3872,7 @@
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr"/>
@@ -3916,7 +3916,7 @@
       </c>
       <c r="I81" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J81" s="5" t="inlineStr">
@@ -3960,7 +3960,7 @@
       <c r="H82" s="2" t="inlineStr"/>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr"/>
@@ -4000,7 +4000,7 @@
       <c r="H83" s="12" t="inlineStr"/>
       <c r="I83" s="12" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J83" s="12" t="inlineStr">
@@ -4044,7 +4044,7 @@
       <c r="H84" s="2" t="inlineStr"/>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr"/>
@@ -4084,7 +4084,7 @@
       <c r="H85" s="5" t="inlineStr"/>
       <c r="I85" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J85" s="5" t="inlineStr"/>
@@ -4124,7 +4124,7 @@
       <c r="H86" s="2" t="inlineStr"/>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr"/>
@@ -4164,7 +4164,7 @@
       <c r="H87" s="5" t="inlineStr"/>
       <c r="I87" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J87" s="5" t="inlineStr"/>
@@ -4204,7 +4204,7 @@
       <c r="H88" s="2" t="inlineStr"/>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr"/>
@@ -4244,7 +4244,7 @@
       <c r="H89" s="5" t="inlineStr"/>
       <c r="I89" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J89" s="5" t="inlineStr"/>
@@ -4288,7 +4288,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -4332,7 +4332,7 @@
       <c r="H91" s="12" t="inlineStr"/>
       <c r="I91" s="12" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J91" s="12" t="inlineStr">
@@ -4376,7 +4376,7 @@
       <c r="H92" s="2" t="inlineStr"/>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr"/>
@@ -4416,7 +4416,7 @@
       <c r="H93" s="5" t="inlineStr"/>
       <c r="I93" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J93" s="5" t="inlineStr"/>
@@ -4456,7 +4456,7 @@
       <c r="H94" s="2" t="inlineStr"/>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr"/>
@@ -4500,7 +4500,7 @@
       </c>
       <c r="I95" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J95" s="5" t="inlineStr">
@@ -4544,7 +4544,7 @@
       <c r="H96" s="2" t="inlineStr"/>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr"/>
@@ -4584,7 +4584,7 @@
       <c r="H97" s="5" t="inlineStr"/>
       <c r="I97" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J97" s="5" t="inlineStr"/>
@@ -4624,7 +4624,7 @@
       <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr"/>
@@ -4664,7 +4664,7 @@
       <c r="H99" s="5" t="inlineStr"/>
       <c r="I99" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J99" s="5" t="inlineStr"/>
@@ -4704,7 +4704,7 @@
       <c r="H100" s="2" t="inlineStr"/>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr"/>
@@ -4748,7 +4748,7 @@
       </c>
       <c r="I101" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J101" s="5" t="inlineStr">
@@ -4792,7 +4792,7 @@
       <c r="H102" s="2" t="inlineStr"/>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr"/>
@@ -4832,7 +4832,7 @@
       <c r="H103" s="5" t="inlineStr"/>
       <c r="I103" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J103" s="5" t="inlineStr"/>
@@ -4872,7 +4872,7 @@
       <c r="H104" s="2" t="inlineStr"/>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr"/>
@@ -4916,7 +4916,7 @@
       </c>
       <c r="I105" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J105" s="5" t="inlineStr">
@@ -4960,7 +4960,7 @@
       <c r="H106" s="2" t="inlineStr"/>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr"/>
@@ -5000,7 +5000,7 @@
       <c r="H107" s="5" t="inlineStr"/>
       <c r="I107" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J107" s="5" t="inlineStr"/>
@@ -5044,7 +5044,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -5088,7 +5088,7 @@
       <c r="H109" s="5" t="inlineStr"/>
       <c r="I109" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J109" s="5" t="inlineStr"/>
@@ -5128,7 +5128,7 @@
       <c r="H110" s="9" t="inlineStr"/>
       <c r="I110" s="9" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J110" s="9" t="inlineStr">
@@ -5172,7 +5172,7 @@
       <c r="H111" s="9" t="inlineStr"/>
       <c r="I111" s="9" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J111" s="9" t="inlineStr">
@@ -5220,7 +5220,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -5264,7 +5264,7 @@
       <c r="H113" s="5" t="inlineStr"/>
       <c r="I113" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J113" s="5" t="inlineStr"/>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -5352,7 +5352,7 @@
       <c r="H115" s="5" t="inlineStr"/>
       <c r="I115" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>MB, GM, DH</t>
         </is>
       </c>
       <c r="J115" s="5" t="inlineStr"/>
@@ -5392,7 +5392,7 @@
       <c r="H116" s="2" t="inlineStr"/>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr"/>
@@ -5432,7 +5432,7 @@
       <c r="H117" s="5" t="inlineStr"/>
       <c r="I117" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J117" s="5" t="inlineStr"/>
@@ -5472,7 +5472,7 @@
       <c r="H118" s="2" t="inlineStr"/>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr"/>
@@ -5516,7 +5516,7 @@
       </c>
       <c r="I119" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J119" s="5" t="inlineStr">
@@ -5560,7 +5560,7 @@
       <c r="H120" s="2" t="inlineStr"/>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr"/>
@@ -5600,7 +5600,7 @@
       <c r="H121" s="12" t="inlineStr"/>
       <c r="I121" s="12" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J121" s="12" t="inlineStr">
@@ -5644,7 +5644,7 @@
       <c r="H122" s="2" t="inlineStr"/>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr"/>
@@ -5684,7 +5684,7 @@
       <c r="H123" s="5" t="inlineStr"/>
       <c r="I123" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J123" s="5" t="inlineStr"/>
@@ -5724,7 +5724,7 @@
       <c r="H124" s="2" t="inlineStr"/>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr"/>
@@ -5764,7 +5764,7 @@
       <c r="H125" s="5" t="inlineStr"/>
       <c r="I125" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J125" s="5" t="inlineStr"/>
@@ -5804,7 +5804,7 @@
       <c r="H126" s="2" t="inlineStr"/>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr"/>
@@ -5844,7 +5844,7 @@
       <c r="H127" s="5" t="inlineStr"/>
       <c r="I127" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J127" s="5" t="inlineStr"/>
@@ -5888,7 +5888,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -5932,7 +5932,7 @@
       <c r="H129" s="12" t="inlineStr"/>
       <c r="I129" s="12" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J129" s="12" t="inlineStr">
@@ -5976,7 +5976,7 @@
       <c r="H130" s="2" t="inlineStr"/>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr"/>
@@ -6016,7 +6016,7 @@
       <c r="H131" s="5" t="inlineStr"/>
       <c r="I131" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J131" s="5" t="inlineStr"/>
@@ -6056,7 +6056,7 @@
       <c r="H132" s="2" t="inlineStr"/>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr"/>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="I133" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J133" s="5" t="inlineStr">
@@ -6144,7 +6144,7 @@
       <c r="H134" s="2" t="inlineStr"/>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr"/>
@@ -6184,7 +6184,7 @@
       <c r="H135" s="5" t="inlineStr"/>
       <c r="I135" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J135" s="5" t="inlineStr"/>
@@ -6224,7 +6224,7 @@
       <c r="H136" s="2" t="inlineStr"/>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr"/>
@@ -6264,7 +6264,7 @@
       <c r="H137" s="5" t="inlineStr"/>
       <c r="I137" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J137" s="5" t="inlineStr"/>
@@ -6304,7 +6304,7 @@
       <c r="H138" s="2" t="inlineStr"/>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr"/>
@@ -6348,7 +6348,7 @@
       </c>
       <c r="I139" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J139" s="5" t="inlineStr">
@@ -6392,7 +6392,7 @@
       <c r="H140" s="2" t="inlineStr"/>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr"/>
@@ -6432,7 +6432,7 @@
       <c r="H141" s="5" t="inlineStr"/>
       <c r="I141" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J141" s="5" t="inlineStr"/>
@@ -6472,7 +6472,7 @@
       <c r="H142" s="2" t="inlineStr"/>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr"/>
@@ -6516,7 +6516,7 @@
       </c>
       <c r="I143" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J143" s="5" t="inlineStr">
@@ -6560,7 +6560,7 @@
       <c r="H144" s="2" t="inlineStr"/>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr"/>
@@ -6600,7 +6600,7 @@
       <c r="H145" s="5" t="inlineStr"/>
       <c r="I145" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J145" s="5" t="inlineStr"/>
@@ -6644,7 +6644,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -6688,7 +6688,7 @@
       <c r="H147" s="5" t="inlineStr"/>
       <c r="I147" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J147" s="5" t="inlineStr"/>
@@ -6728,7 +6728,7 @@
       <c r="H148" s="9" t="inlineStr"/>
       <c r="I148" s="9" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J148" s="9" t="inlineStr">
@@ -6772,7 +6772,7 @@
       <c r="H149" s="9" t="inlineStr"/>
       <c r="I149" s="9" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J149" s="9" t="inlineStr">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -6864,7 +6864,7 @@
       <c r="H151" s="5" t="inlineStr"/>
       <c r="I151" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J151" s="5" t="inlineStr"/>
@@ -6908,7 +6908,7 @@
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -6952,7 +6952,7 @@
       <c r="H153" s="5" t="inlineStr"/>
       <c r="I153" s="5" t="inlineStr">
         <is>
-          <t>JCS</t>
+          <t>DH, GM, VB</t>
         </is>
       </c>
       <c r="J153" s="5" t="inlineStr"/>

</xml_diff>